<commit_message>
Refactor US workbook around nine-part series
</commit_message>
<xml_diff>
--- a/US Markets and Portfolio Construction/US_Markets_Portfolio_Construction_Final_Workbook.xlsx
+++ b/US Markets and Portfolio Construction/US_Markets_Portfolio_Construction_Final_Workbook.xlsx
@@ -2,19 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" r:id="R0a14714deb0e4882"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P1 - Cost of Ownership" sheetId="2" r:id="R0eda23e80b2b4c7f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P1 - NRA Tax" sheetId="3" r:id="Re2701a38b38045db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P2 - Diversification" sheetId="4" r:id="R9c6e3b93ec40435a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P2 - Blended ER" sheetId="5" r:id="R946ebf944a324f8f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P3 - HHI Concentration" sheetId="6" r:id="R9e820396e2684d5d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P4 - Matrix Variance" sheetId="7" r:id="R84497487b3c643ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P4 - Options Wheel" sheetId="8" r:id="R0c26497295854ee1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P4 - Tax Calculators" sheetId="9" r:id="Rcc8c5045d31149d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P5 - Rebalancing" sheetId="10" r:id="Ra6cd266b71d54921"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P5 - DCA vs Lump Sum" sheetId="11" r:id="Rc0981abe752a41d0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P5 - Sequence of Returns" sheetId="12" r:id="Rdae9384d51c9405e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P5 - Case Study" sheetId="13" r:id="Re3f47b59043a4bee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P01 Guide &amp; Map" sheetId="1" r:id="R28c490b2e0544948"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P02 Cost &amp; Ownership" sheetId="2" r:id="Rdc3843b6973f4385"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P03 Cross-Border Tax" sheetId="3" r:id="Rf89d527a34ac4ecc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P04 Diversification" sheetId="4" r:id="R650005b76ebe4479"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P04 Blended Cost" sheetId="5" r:id="Rf2b728030368470c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P05 Core Concentration" sheetId="6" r:id="Rb03bea01f88045cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P06 Portfolio Risk" sheetId="7" r:id="Rb20357c852cd46b6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P07 Options Sleeve" sheetId="8" r:id="Rc28cb5fdb39b406c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P07 Tax &amp; Location" sheetId="9" r:id="R4b7d95a81ee64e47"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P08 Rebalancing" sheetId="10" r:id="Rb9888f5bcddf4fc1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P09 DCA &amp; Contributions" sheetId="11" r:id="R09df6130cd56400c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P09 Sequence Risk" sheetId="12" r:id="R3e94868b61f442ab"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="P09 Full Case Study" sheetId="13" r:id="R7304fa314ead4cd3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -22,120 +22,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <x:sst xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:si>
-    <x:t xml:space="preserve">US Markets and Portfolio Construction — Companion Workbook</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Every calculation table and worked example across the five-part article series, live and editable.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Color legend</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Blue text</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">A supplied input or assumption. Change these — every formula recalculates.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Black text</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">A formula that calculates using only cells on the same worksheet.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Green text</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">A formula that pulls a value from a different worksheet in this workbook.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Yellow fill</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">A key assumption worth double-checking before relying on the sheet.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Sheet index</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">P1 - Cost of Ownership</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Expense-ratio compounding across six vehicles; Part 1, Table 1 and Appendix 1.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">P1 - NRA Tax</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Nonresident-alien dividend withholding and US estate-tax threshold calculators; Part 1 / Appendix 1.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">P2 - Diversification</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Two- and three-asset portfolio variance, with a correlation-sensitivity table; Part 2 / Appendix 2.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">P2 - Blended ER</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Weighted blended expense ratio for a multi-sleeve core-satellite portfolio; Part 2, Table 2.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">P3 - HHI Concentration</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Herfindahl-Hirschman Index and effective-N calculator for up to 30 holdings; Part 3 / Appendix 3.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">P4 - Matrix Variance</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Four-asset portfolio variance in matrix form; Part 4, Equation 4.1 / Appendix 4.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">P4 - Options Wheel</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Cash-secured put and covered-call cycle economics; Part 4, Table 1 / Appendix 4.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">P4 - Tax Calculators</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Qualified-dividend, wash-sale, and 2026 long-term capital-gains bracket calculators; Part 4.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">P5 - Rebalancing</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">One-year drift and the rebalancing trade required to restore target weights; Part 5, Table 2 / Appendix 5.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">P5 - DCA vs Lump Sum</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Lump-sum vs. dollar-cost-averaging comparison under two illustrative return paths; Part 5, Table 1.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">P5 - Sequence of Returns</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Identical average return, reordered, showing the effect of withdrawal timing; Part 5, Table 3 / Appendix 5.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">P5 - Case Study</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Ten-year accumulation projection for the full worked case study; Part 5, Table 4 / Appendix 5.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">All growth-rate, volatility, correlation, and yield figures throughout this workbook are clearly labelled illustrative assumptions for demonstration purposes, matching the corresponding article text — not forecasts, and not personalized financial or tax advice. Expense ratios, statutory tax thresholds, and index-methodology facts are sourced from the primary sources cited in each article's reference list, current as of the 'Accessed' dates shown there.</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Part 1 — Cost of Ownership: Expense-Ratio Compounding</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Change the principal or gross-return assumption below (blue) and every fund's projected value recalculates.</x:t>
   </x:si>
   <x:si>
@@ -196,9 +82,6 @@
     <x:t xml:space="preserve">Gross return</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Part 1 — Nonresident-Alien Withholding and Estate-Tax Thresholds</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">1. Dividend withholding</x:t>
   </x:si>
   <x:si>
@@ -283,9 +166,6 @@
     <x:t xml:space="preserve">Form 706-NA filing required?</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Part 2 — Two-Asset Diversification Mathematics (Equation 2.1)</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Equity weight (w1)</x:t>
   </x:si>
   <x:si>
@@ -358,9 +238,6 @@
     <x:t xml:space="preserve">Three-asset portfolio SD</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Part 2 — Blended Expense Ratio of a Core-Satellite Portfolio</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Total portfolio value ($)</x:t>
   </x:si>
   <x:si>
@@ -418,9 +295,6 @@
     <x:t xml:space="preserve">Blended ER (using expense ratios from the table above)</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Part 3 — Herfindahl-Hirschman Index and Effective-N Calculator</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Paste up to 30 holding weights (as decimals, e.g. 0.08 for 8%) into column B. Unused rows can be left at 0%.</x:t>
   </x:si>
   <x:si>
@@ -469,9 +343,6 @@
     <x:t xml:space="preserve">Effective N</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Part 4 — Four-Asset Portfolio Variance (Equation 4.1: sigma_p^2 = w'.Sigma.w)</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Weights</x:t>
   </x:si>
   <x:si>
@@ -493,18 +364,9 @@
     <x:t xml:space="preserve">Correlation matrix</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Covariance matrix (=vol_i * vol_j * rho_ij)</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Portfolio variance (full double-sum expansion of w'.Sigma.w)</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">The formula in B26 is the full 16-term double sum (4x4) behind Equation 4.1 — algebraically identical to the compact w'.Sigma.w matrix notation used in the article.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Part 4 — Options Wheel: Cash-Secured Put + Covered Call Cycle</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Stage 1: Cash-secured put</x:t>
   </x:si>
   <x:si>
@@ -535,9 +397,6 @@
     <x:t xml:space="preserve">Naive annualized (x12, no compounding, illustrative only)</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Stage 2: If assigned -&gt; covered call</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Effective cost basis after assignment (=B11)</x:t>
   </x:si>
   <x:si>
@@ -589,9 +448,6 @@
     <x:t xml:space="preserve">Period yield on collateral</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Part 4 — Dividend, Wash-Sale, and Capital-Gains Tax Calculators</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">1. Qualified vs. non-qualified dividend</x:t>
   </x:si>
   <x:si>
@@ -691,9 +547,6 @@
     <x:t xml:space="preserve">Effective rate on the gain</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Part 5 — One-Year Drift and the Rebalancing Trade</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Portfolio total ($)</x:t>
   </x:si>
   <x:si>
@@ -736,9 +589,6 @@
     <x:t xml:space="preserve">Net (should be $0 -- a rebalance moves money between sleeves, not in or out)</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Part 5 — Lump Sum vs. Dollar-Cost Averaging, Two Illustrative Paths</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Lump sum amount</x:t>
   </x:si>
   <x:si>
@@ -793,12 +643,6 @@
     <x:t xml:space="preserve">Dip then recover</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Part 5 — Sequence-of-Returns Risk: Same Average Return, Different Order</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Fixed annual withdrawal (not inflation-adjusted, to isolate the sequencing effect)</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Year</x:t>
   </x:si>
   <x:si>
@@ -829,9 +673,6 @@
     <x:t xml:space="preserve">Both retirees experience the identical set of ten annual returns (two -20%/-15% shock years plus eight positive years); only the ORDER differs. Equation 5.1 (Vt = Vt-1 x (1+rt) - W) is applied identically each year -- the divergent outcome comes entirely from where the shock years fall in that sequence, not from any difference in average performance.</x:t>
   </x:si>
   <x:si>
-    <x:t xml:space="preserve">Part 5 — Full Case Study: Ten-Year Accumulation Projection</x:t>
-  </x:si>
-  <x:si>
     <x:t xml:space="preserve">Starting balance</x:t>
   </x:si>
   <x:si>
@@ -854,9 +695,6 @@
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Growth from returns</x:t>
-  </x:si>
-  <x:si>
-    <x:t xml:space="preserve">Approx. annual cost of ownership in year 10 (balance x blended ER)</x:t>
   </x:si>
   <x:si>
     <x:t xml:space="preserve">Rows 10-129 (hidden detail) run the month-by-month compounding formula (Equation 5.3) for all 120 months; the year-end summary above pulls the balance at the end of each 12th month. Change the starting balance, monthly contribution, or return assumption in B3:B5 and every downstream figure recalculates, including the blended-ER figure pulled live from the 'P2 - Blended ER' worksheet.</x:t>
@@ -878,7 +716,7 @@
     <x:numFmt numFmtId="172" formatCode="0.0"/>
     <x:numFmt numFmtId="173" formatCode="0.0000%"/>
   </x:numFmts>
-  <x:fonts count="12">
+  <x:fonts count="23">
     <x:font>
       <x:sz val="11"/>
       <x:color theme="1"/>
@@ -940,8 +778,73 @@
       <x:color rgb="FFFFFFFF"/>
       <x:name val="Arial"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF17365D"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF404040"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF404040"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:i/>
+      <x:sz val="9"/>
+      <x:color rgb="FF404040"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="15"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:sz val="11"/>
+      <x:color rgb="FF404040"/>
+      <x:name val="Calibri"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF404040"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF666666"/>
+      <x:name val="Arial"/>
+    </x:font>
+    <x:font>
+      <x:i/>
+      <x:sz val="10"/>
+      <x:color rgb="FF666666"/>
+      <x:name val="Calibri"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="9">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -956,6 +859,31 @@
     <x:fill>
       <x:patternFill patternType="solid">
         <x:fgColor rgb="FF305496"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFD9EAF7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF2F8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF17365D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF2F2F2"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -1001,7 +929,7 @@
     <x:xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <x:xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="1" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="56">
+  <x:cellXfs count="91">
     <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
     </x:xf>
@@ -1169,6 +1097,111 @@
     </x:xf>
     <x:xf numFmtId="167" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="4" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="13" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="6" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="7" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="8" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="14" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="13" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="14" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="13" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="17" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="13" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="12" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="18" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="10" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="21" fillId="8" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="22" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="22" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="22" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="6">
@@ -1419,192 +1452,244 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF1F4E78"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="38" style="1" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="70" style="1" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="42" style="1" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="76" style="1" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1" ht="17.350000381469727" hidden="0">
-      <x:c r="A1" s="2" t="s">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="B1" s="2"/>
+    <x:row r="1" ht="48" hidden="0" customHeight="1">
+      <x:c r="A1" s="80" t="str">
+        <x:v>US Markets and Portfolio Construction</x:v>
+      </x:c>
+      <x:c r="B1" s="80" t="str">
+        <x:v>Nine-Part Companion Workbook</x:v>
+      </x:c>
       <x:c r="C1" s="2"/>
       <x:c r="D1" s="2"/>
       <x:c r="E1" s="2"/>
       <x:c r="F1" s="2"/>
     </x:row>
-    <x:row r="2" ht="15" hidden="0">
-      <x:c r="A2" s="3" t="s">
-        <x:v>1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4" ht="15" hidden="0">
-      <x:c r="A4" s="4" t="s">
-        <x:v>2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5" ht="15" hidden="0">
-      <x:c r="A5" s="5" t="s">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="B5" s="6" t="s">
-        <x:v>4</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="6" ht="15" hidden="0">
-      <x:c r="A6" s="1" t="s">
-        <x:v>5</x:v>
-      </x:c>
-      <x:c r="B6" s="1" t="s">
-        <x:v>6</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7" ht="15" hidden="0">
-      <x:c r="A7" s="7" t="s">
-        <x:v>7</x:v>
-      </x:c>
-      <x:c r="B7" s="6" t="s">
-        <x:v>8</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8" ht="15" hidden="0">
-      <x:c r="A8" s="8" t="s">
-        <x:v>9</x:v>
-      </x:c>
-      <x:c r="B8" s="6" t="s">
-        <x:v>10</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="10" ht="15" hidden="0">
-      <x:c r="A10" s="4" t="s">
-        <x:v>11</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="11" ht="26.850000381469727" hidden="0">
-      <x:c r="A11" s="4" t="s">
-        <x:v>12</x:v>
-      </x:c>
-      <x:c r="B11" s="9" t="s">
-        <x:v>13</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="12" ht="26.850000381469727" hidden="0">
-      <x:c r="A12" s="4" t="s">
-        <x:v>14</x:v>
-      </x:c>
-      <x:c r="B12" s="9" t="s">
-        <x:v>15</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="13" ht="26.850000381469727" hidden="0">
-      <x:c r="A13" s="4" t="s">
-        <x:v>16</x:v>
-      </x:c>
-      <x:c r="B13" s="9" t="s">
-        <x:v>17</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="14" ht="26.850000381469727" hidden="0">
-      <x:c r="A14" s="4" t="s">
-        <x:v>18</x:v>
-      </x:c>
-      <x:c r="B14" s="9" t="s">
-        <x:v>19</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="15" ht="26.850000381469727" hidden="0">
-      <x:c r="A15" s="4" t="s">
-        <x:v>20</x:v>
-      </x:c>
-      <x:c r="B15" s="9" t="s">
-        <x:v>21</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16" ht="26.850000381469727" hidden="0">
-      <x:c r="A16" s="4" t="s">
-        <x:v>22</x:v>
-      </x:c>
-      <x:c r="B16" s="9" t="s">
-        <x:v>23</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17" ht="26.850000381469727" hidden="0">
-      <x:c r="A17" s="4" t="s">
-        <x:v>24</x:v>
-      </x:c>
-      <x:c r="B17" s="9" t="s">
-        <x:v>25</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18" ht="26.850000381469727" hidden="0">
-      <x:c r="A18" s="4" t="s">
-        <x:v>26</x:v>
-      </x:c>
-      <x:c r="B18" s="9" t="s">
-        <x:v>27</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19" ht="26.850000381469727" hidden="0">
-      <x:c r="A19" s="4" t="s">
-        <x:v>28</x:v>
-      </x:c>
-      <x:c r="B19" s="9" t="s">
-        <x:v>29</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20" ht="26.850000381469727" hidden="0">
-      <x:c r="A20" s="4" t="s">
-        <x:v>30</x:v>
-      </x:c>
-      <x:c r="B20" s="9" t="s">
-        <x:v>31</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21" ht="26.850000381469727" hidden="0">
-      <x:c r="A21" s="4" t="s">
-        <x:v>32</x:v>
-      </x:c>
-      <x:c r="B21" s="9" t="s">
-        <x:v>33</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="22" ht="26.850000381469727" hidden="0">
-      <x:c r="A22" s="4" t="s">
-        <x:v>34</x:v>
-      </x:c>
-      <x:c r="B22" s="9" t="s">
-        <x:v>35</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25" ht="60" hidden="0" customHeight="1">
-      <x:c r="A25" s="10" t="s">
-        <x:v>36</x:v>
-      </x:c>
-      <x:c r="B25" s="10"/>
+    <x:row r="2" ht="34" hidden="0" customHeight="1">
+      <x:c r="A2" s="3" t="str">
+        <x:v>Purpose</x:v>
+      </x:c>
+      <x:c r="B2" s="75" t="str">
+        <x:v>Use this workbook with the unified nine-part research series. Blue input cells remain editable; formula cells recalculate portfolio, tax, contribution and withdrawal examples.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3" ht="34" customHeight="1">
+      <x:c r="A3" s="61" t="str">
+        <x:v>Part</x:v>
+      </x:c>
+      <x:c r="B3" s="76" t="str">
+        <x:v>Workbook coverage</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="34" hidden="0" customHeight="1">
+      <x:c r="A4" s="68" t="str">
+        <x:v>Part 01: Foundations</x:v>
+      </x:c>
+      <x:c r="B4" s="75" t="str">
+        <x:v>This guide provides the decision sequence and maps every model to the research progression.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="34" hidden="0" customHeight="1">
+      <x:c r="A5" s="68" t="str">
+        <x:v>Part 02: Cost and ownership</x:v>
+      </x:c>
+      <x:c r="B5" s="75" t="str">
+        <x:v>P02 Cost &amp; Ownership models expense-ratio compounding across investment vehicles.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="34" hidden="0" customHeight="1">
+      <x:c r="A6" s="69" t="str">
+        <x:v>Part 03: Cross-border access</x:v>
+      </x:c>
+      <x:c r="B6" s="75" t="str">
+        <x:v>P03 Cross-Border Tax models withholding and nonresident estate-tax exposure.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" ht="34" hidden="0" customHeight="1">
+      <x:c r="A7" s="68" t="str">
+        <x:v>Part 04: Portfolio architecture</x:v>
+      </x:c>
+      <x:c r="B7" s="75" t="str">
+        <x:v>P04 Diversification and P04 Blended Cost model variance, correlation and blended expense ratios.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="34" hidden="0" customHeight="1">
+      <x:c r="A8" s="69" t="str">
+        <x:v>Part 05: Core construction</x:v>
+      </x:c>
+      <x:c r="B8" s="75" t="str">
+        <x:v>P05 Core Concentration measures overlap and concentration using the Herfindahl-Hirschman Index.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="34" customHeight="1">
+      <x:c r="A9" s="69" t="str">
+        <x:v>Part 06: Satellite exposure</x:v>
+      </x:c>
+      <x:c r="B9" s="75" t="str">
+        <x:v>P06 Portfolio Risk calculates covariance-matrix portfolio variance for multi-asset and satellite allocations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="34" hidden="0" customHeight="1">
+      <x:c r="A10" s="68" t="str">
+        <x:v>Part 07: Tactical sleeves and tax</x:v>
+      </x:c>
+      <x:c r="B10" s="75" t="str">
+        <x:v>P07 Options Sleeve and P07 Tax &amp; Location model an options cycle, dividend tax, wash sales and capital-gains brackets.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="34" hidden="0" customHeight="1">
+      <x:c r="A11" s="68" t="str">
+        <x:v>Part 08: Governance</x:v>
+      </x:c>
+      <x:c r="B11" s="77" t="str">
+        <x:v>P08 Rebalancing compares drift, threshold rules and disciplined portfolio maintenance.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="34" hidden="0" customHeight="1">
+      <x:c r="A12" s="68" t="str">
+        <x:v>Part 09: Funding and withdrawals</x:v>
+      </x:c>
+      <x:c r="B12" s="77" t="str">
+        <x:v>P09 DCA &amp; Contributions, P09 Sequence Risk and P09 Full Case Study connect contributions, rebalancing, fees and withdrawals.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="13" ht="34" hidden="0" customHeight="1">
+      <x:c r="A13" s="73" t="str">
+        <x:v>Progression</x:v>
+      </x:c>
+      <x:c r="B13" s="77" t="str">
+        <x:v>Foundation → ownership route → portfolio architecture → core → satellites → implementation → governance → lifecycle.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="14" ht="34" hidden="0" customHeight="1">
+      <x:c r="A14" s="73" t="str">
+        <x:v>Workbook relationship</x:v>
+      </x:c>
+      <x:c r="B14" s="77" t="str">
+        <x:v>The sheets complement the articles. They expose assumptions and calculations without replacing the written discussion, evidence or cited limitations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15" ht="34" hidden="0" customHeight="1">
+      <x:c r="A15" s="73" t="str">
+        <x:v>Input convention</x:v>
+      </x:c>
+      <x:c r="B15" s="77" t="str">
+        <x:v>Blue cells are user inputs. Change one assumption at a time and review the linked outputs.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16" ht="34" hidden="0" customHeight="1">
+      <x:c r="A16" s="73" t="str">
+        <x:v>Formula convention</x:v>
+      </x:c>
+      <x:c r="B16" s="77" t="str">
+        <x:v>Green cells contain formulas. Do not overwrite them unless you are intentionally adapting the model.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17" ht="34" hidden="0" customHeight="1">
+      <x:c r="A17" s="73" t="str">
+        <x:v>Output convention</x:v>
+      </x:c>
+      <x:c r="B17" s="77" t="str">
+        <x:v>Orange cells highlight decision outputs and scenario comparisons.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18" ht="34" hidden="0" customHeight="1">
+      <x:c r="A18" s="73" t="str">
+        <x:v>Units</x:v>
+      </x:c>
+      <x:c r="B18" s="77" t="str">
+        <x:v>Dollar amounts are in USD unless a worksheet states otherwise. Percentages are stored as numeric rates.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19" ht="34" hidden="0" customHeight="1">
+      <x:c r="A19" s="73" t="str">
+        <x:v>Tax scope</x:v>
+      </x:c>
+      <x:c r="B19" s="77" t="str">
+        <x:v>Tax sheets are educational illustrations. Verify current rules, residence, treaty position and account structure before acting.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20" ht="34" hidden="0" customHeight="1">
+      <x:c r="A20" s="73" t="str">
+        <x:v>Risk scope</x:v>
+      </x:c>
+      <x:c r="B20" s="77" t="str">
+        <x:v>Portfolio examples illustrate mechanics. They do not forecast returns or guarantee diversification benefits.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21" ht="34" hidden="0" customHeight="1">
+      <x:c r="A21" s="73" t="str">
+        <x:v>Source trace</x:v>
+      </x:c>
+      <x:c r="B21" s="77" t="str">
+        <x:v>The reconciled source history and superseded workbook checksums are recorded in WORKBOOK_LINEAGE.md beside this file.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="34" hidden="0" customHeight="1">
+      <x:c r="A22" s="73" t="str">
+        <x:v>Canonical release</x:v>
+      </x:c>
+      <x:c r="B22" s="77" t="str">
+        <x:v>This workbook is the authoritative companion for the nine-part unified US Markets and Portfolio Construction series.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23" ht="34" customHeight="1">
+      <x:c r="A23" s="74" t="str">
+        <x:v>Series structure</x:v>
+      </x:c>
+      <x:c r="B23" s="75" t="str">
+        <x:v>All nine parts are visible in the tab names, with additional tabs only where a part contains distinct calculations.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24" ht="34" customHeight="1">
+      <x:c r="A24" s="74" t="str">
+        <x:v>Recommended use</x:v>
+      </x:c>
+      <x:c r="B24" s="81" t="str">
+        <x:v>Read each article first, then use the matching worksheet to test assumptions and reproduce the worked examples.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25" ht="34" hidden="0" customHeight="1">
+      <x:c r="A25" s="72" t="str">
+        <x:v>Version</x:v>
+      </x:c>
+      <x:c r="B25" s="82" t="str">
+        <x:v>Nine-part presentation refactor, 16 September 2026</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
-  <x:mergeCells>
-    <x:mergeCell ref="A1:F1"/>
-    <x:mergeCell ref="A25:B25"/>
-  </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFA5A5A5"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" style="1" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="34" style="1" hidden="0" customWidth="1"/>
     <x:col min="2" max="3" width="14" style="1" hidden="0" customWidth="1"/>
     <x:col min="4" max="6" width="16" style="1" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="18" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="17.350000381469727" hidden="0">
-      <x:c r="A1" s="2" t="s">
-        <x:v>223</x:v>
+      <x:c r="A1" s="2" t="str">
+        <x:v>Part 08: Rebalancing and Portfolio Governance</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -1614,7 +1699,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0">
       <x:c r="A2" s="1" t="s">
-        <x:v>224</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="B2" s="12" t="n">
         <x:v>50000</x:v>
@@ -1622,27 +1707,27 @@
     </x:row>
     <x:row r="3" ht="39.54999923706055" hidden="0">
       <x:c r="A3" s="14" t="s">
-        <x:v>114</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="B3" s="14" t="s">
-        <x:v>225</x:v>
+        <x:v>176</x:v>
       </x:c>
       <x:c r="C3" s="14" t="s">
-        <x:v>226</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="D3" s="14" t="s">
-        <x:v>227</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="E3" s="14" t="s">
-        <x:v>228</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="F3" s="14" t="s">
-        <x:v>229</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0">
       <x:c r="A4" s="15" t="s">
-        <x:v>230</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="B4" s="20" t="n">
         <x:v>0.55</x:v>
@@ -1665,7 +1750,7 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0">
       <x:c r="A5" s="15" t="s">
-        <x:v>127</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="B5" s="20" t="n">
         <x:v>0.15</x:v>
@@ -1688,7 +1773,7 @@
     </x:row>
     <x:row r="6" ht="15" hidden="0">
       <x:c r="A6" s="15" t="s">
-        <x:v>128</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="B6" s="20" t="n">
         <x:v>0.15</x:v>
@@ -1711,7 +1796,7 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0">
       <x:c r="A7" s="15" t="s">
-        <x:v>154</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="B7" s="20" t="n">
         <x:v>0.15</x:v>
@@ -1734,7 +1819,7 @@
     </x:row>
     <x:row r="8" ht="15" hidden="0">
       <x:c r="A8" s="35" t="s">
-        <x:v>122</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="B8" s="22"/>
       <x:c r="C8" s="22"/>
@@ -1750,7 +1835,7 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0">
       <x:c r="A11" s="19" t="s">
-        <x:v>231</x:v>
+        <x:v>182</x:v>
       </x:c>
       <x:c r="B11" s="19"/>
       <x:c r="C11" s="19"/>
@@ -1760,27 +1845,27 @@
     </x:row>
     <x:row r="12" ht="26.850000381469727" hidden="0">
       <x:c r="A12" s="14" t="s">
-        <x:v>114</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="B12" s="14" t="s">
-        <x:v>232</x:v>
+        <x:v>183</x:v>
       </x:c>
       <x:c r="C12" s="14" t="s">
-        <x:v>233</x:v>
+        <x:v>184</x:v>
       </x:c>
       <x:c r="D12" s="14" t="s">
-        <x:v>234</x:v>
+        <x:v>185</x:v>
       </x:c>
       <x:c r="E12" s="14" t="s">
-        <x:v>235</x:v>
+        <x:v>186</x:v>
       </x:c>
       <x:c r="F12" s="14" t="s">
-        <x:v>236</x:v>
+        <x:v>187</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0">
       <x:c r="A13" s="15" t="s">
-        <x:v>230</x:v>
+        <x:v>181</x:v>
       </x:c>
       <x:c r="B13" s="51" t="n">
         <x:f aca="0">E4</x:f>
@@ -1805,7 +1890,7 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0">
       <x:c r="A14" s="15" t="s">
-        <x:v>127</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="B14" s="51" t="n">
         <x:f aca="0">E5</x:f>
@@ -1830,7 +1915,7 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0">
       <x:c r="A15" s="15" t="s">
-        <x:v>128</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="B15" s="51" t="n">
         <x:f aca="0">E6</x:f>
@@ -1855,7 +1940,7 @@
     </x:row>
     <x:row r="16" ht="15" hidden="0">
       <x:c r="A16" s="15" t="s">
-        <x:v>154</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="B16" s="51" t="n">
         <x:f aca="0">E7</x:f>
@@ -1879,9 +1964,12 @@
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0">
-      <x:c r="A17" s="11" t="s">
-        <x:v>237</x:v>
-      </x:c>
+      <x:c r="A17" s="77" t="s">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="B17" s="75"/>
+      <x:c r="C17" s="75"/>
+      <x:c r="D17" s="75"/>
       <x:c r="E17" s="28" t="n">
         <x:f aca="0">SUM(E13:E16)</x:f>
         <x:v>3.637978807091713e-12</x:v>
@@ -1891,6 +1979,7 @@
   <x:mergeCells>
     <x:mergeCell ref="A1:F1"/>
     <x:mergeCell ref="A11:F11"/>
+    <x:mergeCell ref="A17:D17"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -1898,16 +1987,22 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF8064A2"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="20" style="1" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" style="1" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="48" style="1" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22" style="1" hidden="0" customWidth="1"/>
     <x:col min="3" max="4" width="16" style="1" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="22" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="22" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="17.350000381469727" hidden="0">
-      <x:c r="A1" s="2" t="s">
-        <x:v>238</x:v>
+      <x:c r="A1" s="2" t="str">
+        <x:v>Part 09: Contributions and Dollar-Cost Averaging</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -1915,19 +2010,19 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0" customHeight="1">
       <x:c r="A3" s="1" t="s">
-        <x:v>239</x:v>
+        <x:v>189</x:v>
       </x:c>
       <x:c r="B3" s="12" t="n">
         <x:v>6000</x:v>
       </x:c>
       <x:c r="C3" s="10" t="s">
-        <x:v>240</x:v>
+        <x:v>190</x:v>
       </x:c>
       <x:c r="D3" s="10"/>
     </x:row>
     <x:row r="4" ht="15" hidden="0">
       <x:c r="A4" s="1" t="s">
-        <x:v>241</x:v>
+        <x:v>191</x:v>
       </x:c>
       <x:c r="B4" s="12" t="n">
         <x:v>500</x:v>
@@ -1937,13 +2032,13 @@
     </x:row>
     <x:row r="6" ht="39.54999923706055" hidden="0">
       <x:c r="A6" s="14" t="s">
-        <x:v>242</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="B6" s="14" t="s">
-        <x:v>243</x:v>
+        <x:v>193</x:v>
       </x:c>
       <x:c r="C6" s="14" t="s">
-        <x:v>244</x:v>
+        <x:v>194</x:v>
       </x:c>
       <x:c r="D6" s="14"/>
       <x:c r="E6" s="14"/>
@@ -2082,7 +2177,7 @@
     </x:row>
     <x:row r="20" ht="15" hidden="0">
       <x:c r="A20" s="4" t="s">
-        <x:v>245</x:v>
+        <x:v>195</x:v>
       </x:c>
       <x:c r="B20" s="28" t="n">
         <x:f aca="0">$B$3*(1+B7)*(1+B8)*(1+B9)*(1+B10)*(1+B11)*(1+B12)*(1+B13)*(1+B14)*(1+B15)*(1+B16)*(1+B17)*(1+B18)</x:f>
@@ -2091,7 +2186,7 @@
     </x:row>
     <x:row r="21" ht="15" hidden="0">
       <x:c r="A21" s="4" t="s">
-        <x:v>246</x:v>
+        <x:v>196</x:v>
       </x:c>
       <x:c r="B21" s="28" t="n">
         <x:f aca="0">$B$3*(1+C7)*(1+C8)*(1+C9)*(1+C10)*(1+C11)*(1+C12)*(1+C13)*(1+C14)*(1+C15)*(1+C16)*(1+C17)*(1+C18)</x:f>
@@ -2100,18 +2195,18 @@
     </x:row>
     <x:row r="23" ht="15" hidden="0">
       <x:c r="A23" s="4" t="s">
-        <x:v>247</x:v>
+        <x:v>197</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="39.54999923706055" hidden="0">
       <x:c r="A24" s="14" t="s">
-        <x:v>242</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="B24" s="14" t="s">
-        <x:v>248</x:v>
+        <x:v>198</x:v>
       </x:c>
       <x:c r="C24" s="14" t="s">
-        <x:v>249</x:v>
+        <x:v>199</x:v>
       </x:c>
       <x:c r="D24" s="14"/>
       <x:c r="E24" s="14"/>
@@ -2274,26 +2369,26 @@
     </x:row>
     <x:row r="38" ht="15" hidden="0">
       <x:c r="A38" s="4" t="s">
-        <x:v>250</x:v>
+        <x:v>200</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="26.850000381469727" hidden="0">
       <x:c r="A39" s="14" t="s">
-        <x:v>251</x:v>
+        <x:v>201</x:v>
       </x:c>
       <x:c r="B39" s="14" t="s">
-        <x:v>252</x:v>
+        <x:v>202</x:v>
       </x:c>
       <x:c r="C39" s="14" t="s">
-        <x:v>253</x:v>
+        <x:v>203</x:v>
       </x:c>
       <x:c r="D39" s="14" t="s">
-        <x:v>254</x:v>
+        <x:v>204</x:v>
       </x:c>
     </x:row>
     <x:row r="40" ht="15" hidden="0">
       <x:c r="A40" s="15" t="s">
-        <x:v>255</x:v>
+        <x:v>205</x:v>
       </x:c>
       <x:c r="B40" s="51" t="n">
         <x:f aca="0">B20</x:f>
@@ -2310,7 +2405,7 @@
     </x:row>
     <x:row r="41" ht="15" hidden="0">
       <x:c r="A41" s="15" t="s">
-        <x:v>256</x:v>
+        <x:v>206</x:v>
       </x:c>
       <x:c r="B41" s="51" t="n">
         <x:f aca="0">B21</x:f>
@@ -2336,18 +2431,21 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF8064A2"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10" style="1" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" style="1" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="16" style="1" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" style="1" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="16" style="1" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="52" style="1" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="20" style="1" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="20" style="1" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="20" style="1" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="20" style="1" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="17.350000381469727" hidden="0">
-      <x:c r="A1" s="2" t="s">
-        <x:v>257</x:v>
+      <x:c r="A1" s="2" t="str">
+        <x:v>Part 09: Withdrawal Timing and Sequence Risk</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -2356,15 +2454,15 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0">
       <x:c r="A3" s="1" t="s">
-        <x:v>227</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="B3" s="12" t="n">
         <x:v>1000000</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0">
-      <x:c r="A4" s="53" t="s">
-        <x:v>258</x:v>
+      <x:c r="A4" s="53" t="str">
+        <x:v>Fixed annual withdrawal, not adjusted for inflation</x:v>
       </x:c>
       <x:c r="B4" s="12" t="n">
         <x:v>45000</x:v>
@@ -2375,19 +2473,19 @@
     </x:row>
     <x:row r="7" ht="39.54999923706055" hidden="0">
       <x:c r="A7" s="14" t="s">
-        <x:v>259</x:v>
+        <x:v>207</x:v>
       </x:c>
       <x:c r="B7" s="14" t="s">
-        <x:v>260</x:v>
+        <x:v>208</x:v>
       </x:c>
       <x:c r="C7" s="14" t="s">
-        <x:v>261</x:v>
+        <x:v>209</x:v>
       </x:c>
       <x:c r="D7" s="14" t="s">
-        <x:v>262</x:v>
+        <x:v>210</x:v>
       </x:c>
       <x:c r="E7" s="14" t="s">
-        <x:v>263</x:v>
+        <x:v>211</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0">
@@ -2597,7 +2695,7 @@
     </x:row>
     <x:row r="20" ht="15" hidden="0">
       <x:c r="A20" s="11" t="s">
-        <x:v>264</x:v>
+        <x:v>212</x:v>
       </x:c>
       <x:c r="B20" s="34" t="n">
         <x:f aca="0">AVERAGE(B9:B18)</x:f>
@@ -2608,55 +2706,58 @@
         <x:v>0.03300000000000001</x:v>
       </x:c>
     </x:row>
-    <x:row r="21" ht="15" hidden="0">
-      <x:c r="A21" s="4" t="s">
-        <x:v>265</x:v>
-      </x:c>
+    <x:row r="21" ht="34" hidden="0" customHeight="1">
+      <x:c r="A21" s="90" t="s">
+        <x:v>213</x:v>
+      </x:c>
+      <x:c r="B21" s="75"/>
       <x:c r="C21" s="28" t="n">
         <x:f aca="0">C18</x:f>
         <x:v>666446.2421543258</x:v>
       </x:c>
     </x:row>
-    <x:row r="22" ht="15" hidden="0">
-      <x:c r="A22" s="4" t="s">
-        <x:v>266</x:v>
-      </x:c>
+    <x:row r="22" ht="34" hidden="0" customHeight="1">
+      <x:c r="A22" s="90" t="s">
+        <x:v>214</x:v>
+      </x:c>
+      <x:c r="B22" s="75"/>
       <x:c r="E22" s="28" t="n">
         <x:f aca="0">E18</x:f>
         <x:v>895643.3631130203</x:v>
       </x:c>
     </x:row>
-    <x:row r="23" ht="15" hidden="0">
-      <x:c r="A23" s="4" t="s">
-        <x:v>267</x:v>
-      </x:c>
+    <x:row r="23" ht="34" hidden="0" customHeight="1">
+      <x:c r="A23" s="90" t="s">
+        <x:v>215</x:v>
+      </x:c>
+      <x:c r="B23" s="75"/>
       <x:c r="C23" s="28" t="n">
         <x:f aca="0">E18-C18</x:f>
         <x:v>229197.1209586945</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0" customHeight="1">
-      <x:c r="A25" s="10" t="s">
-        <x:v>268</x:v>
-      </x:c>
-      <x:c r="B25" s="10"/>
-      <x:c r="C25" s="10"/>
-      <x:c r="D25" s="10"/>
-      <x:c r="E25" s="10"/>
+      <x:c r="A25" s="78" t="s">
+        <x:v>216</x:v>
+      </x:c>
+      <x:c r="B25" s="78"/>
+      <x:c r="C25" s="78"/>
+      <x:c r="D25" s="78"/>
+      <x:c r="E25" s="78"/>
     </x:row>
     <x:row r="26" ht="15" hidden="0">
-      <x:c r="A26" s="10"/>
-      <x:c r="B26" s="10"/>
-      <x:c r="C26" s="10"/>
-      <x:c r="D26" s="10"/>
-      <x:c r="E26" s="10"/>
+      <x:c r="A26" s="78"/>
+      <x:c r="B26" s="78"/>
+      <x:c r="C26" s="78"/>
+      <x:c r="D26" s="78"/>
+      <x:c r="E26" s="78"/>
     </x:row>
     <x:row r="27" ht="15" hidden="0">
-      <x:c r="A27" s="10"/>
-      <x:c r="B27" s="10"/>
-      <x:c r="C27" s="10"/>
-      <x:c r="D27" s="10"/>
-      <x:c r="E27" s="10"/>
+      <x:c r="A27" s="78"/>
+      <x:c r="B27" s="78"/>
+      <x:c r="C27" s="78"/>
+      <x:c r="D27" s="78"/>
+      <x:c r="E27" s="78"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -2670,17 +2771,20 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF8064A2"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="14" style="1" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="16" style="1" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="18" style="1" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="16" style="1" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="52" style="1" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="21" style="1" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="21" style="1" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="21" style="1" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="17.350000381469727" hidden="0">
-      <x:c r="A1" s="2" t="s">
-        <x:v>269</x:v>
+      <x:c r="A1" s="2" t="str">
+        <x:v>Part 09: Full Lifecycle Case Study</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -2688,7 +2792,7 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0">
       <x:c r="A3" s="1" t="s">
-        <x:v>270</x:v>
+        <x:v>217</x:v>
       </x:c>
       <x:c r="B3" s="12" t="n">
         <x:v>50000</x:v>
@@ -2696,7 +2800,7 @@
     </x:row>
     <x:row r="4" ht="15" hidden="0">
       <x:c r="A4" s="1" t="s">
-        <x:v>271</x:v>
+        <x:v>218</x:v>
       </x:c>
       <x:c r="B4" s="12" t="n">
         <x:v>500</x:v>
@@ -2724,19 +2828,19 @@
         <x:v>Blended expense ratio (growth-oriented variant)</x:v>
       </x:c>
       <x:c r="B7" s="55" t="n">
-        <x:f aca="0">'P2 - Blended ER'!C22</x:f>
+        <x:f aca="0">'P04 Blended Cost'!C22</x:f>
         <x:v>0.00095</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="26.850000381469727" hidden="0">
       <x:c r="A9" s="14" t="s">
-        <x:v>242</x:v>
+        <x:v>192</x:v>
       </x:c>
       <x:c r="B9" s="14" t="s">
-        <x:v>272</x:v>
+        <x:v>219</x:v>
       </x:c>
       <x:c r="C9" s="14" t="s">
-        <x:v>273</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="D9" s="14"/>
     </x:row>
@@ -4302,21 +4406,21 @@
     </x:row>
     <x:row r="131" ht="15" hidden="0">
       <x:c r="A131" s="4" t="s">
-        <x:v>274</x:v>
+        <x:v>221</x:v>
       </x:c>
     </x:row>
     <x:row r="132" ht="26.850000381469727" hidden="0">
       <x:c r="A132" s="14" t="s">
-        <x:v>275</x:v>
+        <x:v>222</x:v>
       </x:c>
       <x:c r="B132" s="14" t="s">
-        <x:v>276</x:v>
+        <x:v>223</x:v>
       </x:c>
       <x:c r="C132" s="14" t="s">
-        <x:v>273</x:v>
+        <x:v>220</x:v>
       </x:c>
       <x:c r="D132" s="14" t="s">
-        <x:v>277</x:v>
+        <x:v>224</x:v>
       </x:c>
     </x:row>
     <x:row r="133" ht="15" hidden="0">
@@ -4490,8 +4594,8 @@
       </x:c>
     </x:row>
     <x:row r="144" ht="15" hidden="0">
-      <x:c r="A144" s="11" t="s">
-        <x:v>278</x:v>
+      <x:c r="A144" s="11" t="str">
+        <x:v>Annual cost of ownership in year 10</x:v>
       </x:c>
       <x:c r="B144" s="28" t="n">
         <x:f aca="0">B142*B7</x:f>
@@ -4499,24 +4603,24 @@
       </x:c>
     </x:row>
     <x:row r="146" ht="15" hidden="0" customHeight="1">
-      <x:c r="A146" s="10" t="s">
-        <x:v>279</x:v>
-      </x:c>
-      <x:c r="B146" s="10"/>
-      <x:c r="C146" s="10"/>
-      <x:c r="D146" s="10"/>
+      <x:c r="A146" s="78" t="s">
+        <x:v>225</x:v>
+      </x:c>
+      <x:c r="B146" s="78"/>
+      <x:c r="C146" s="78"/>
+      <x:c r="D146" s="78"/>
     </x:row>
     <x:row r="147" ht="15" hidden="0">
-      <x:c r="A147" s="10"/>
-      <x:c r="B147" s="10"/>
-      <x:c r="C147" s="10"/>
-      <x:c r="D147" s="10"/>
+      <x:c r="A147" s="78"/>
+      <x:c r="B147" s="78"/>
+      <x:c r="C147" s="78"/>
+      <x:c r="D147" s="78"/>
     </x:row>
     <x:row r="148" ht="15" hidden="0">
-      <x:c r="A148" s="10"/>
-      <x:c r="B148" s="10"/>
-      <x:c r="C148" s="10"/>
-      <x:c r="D148" s="10"/>
+      <x:c r="A148" s="78"/>
+      <x:c r="B148" s="78"/>
+      <x:c r="C148" s="78"/>
+      <x:c r="D148" s="78"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>
@@ -4529,6 +4633,9 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF2F75B5"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="30" style="1" hidden="0" customWidth="1"/>
@@ -4538,8 +4645,8 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="17.350000381469727" hidden="0">
-      <x:c r="A1" s="2" t="s">
-        <x:v>37</x:v>
+      <x:c r="A1" s="2" t="str">
+        <x:v>Part 02: Wrapper Costs and Long-Term Ownership</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -4550,7 +4657,7 @@
     </x:row>
     <x:row r="2" ht="15" hidden="0" customHeight="1">
       <x:c r="A2" s="10" t="s">
-        <x:v>38</x:v>
+        <x:v>0</x:v>
       </x:c>
       <x:c r="B2" s="10"/>
       <x:c r="C2" s="10"/>
@@ -4561,13 +4668,13 @@
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="11" t="s">
-        <x:v>39</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="B4" s="12" t="n">
         <x:v>10000</x:v>
       </x:c>
       <x:c r="D4" s="10" t="s">
-        <x:v>40</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="E4" s="10"/>
       <x:c r="F4" s="10"/>
@@ -4575,7 +4682,7 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0">
       <x:c r="A5" s="11" t="s">
-        <x:v>41</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="B5" s="13" t="n">
         <x:v>0.08</x:v>
@@ -4587,30 +4694,30 @@
     </x:row>
     <x:row r="7" ht="26.850000381469727" hidden="0">
       <x:c r="A7" s="14" t="s">
-        <x:v>42</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="B7" s="14" t="s">
-        <x:v>43</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="C7" s="14" t="s">
-        <x:v>44</x:v>
+        <x:v>6</x:v>
       </x:c>
       <x:c r="D7" s="14" t="s">
-        <x:v>45</x:v>
+        <x:v>7</x:v>
       </x:c>
       <x:c r="E7" s="14" t="s">
-        <x:v>46</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="F7" s="14" t="s">
-        <x:v>47</x:v>
+        <x:v>9</x:v>
       </x:c>
       <x:c r="G7" s="14" t="s">
-        <x:v>48</x:v>
+        <x:v>10</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="15" hidden="0">
       <x:c r="A8" s="15" t="s">
-        <x:v>49</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="B8" s="16" t="n">
         <x:v>0.0002</x:v>
@@ -4638,7 +4745,7 @@
     </x:row>
     <x:row r="9" ht="15" hidden="0">
       <x:c r="A9" s="15" t="s">
-        <x:v>50</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="B9" s="16" t="n">
         <x:v>0.0003</x:v>
@@ -4666,7 +4773,7 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0">
       <x:c r="A10" s="15" t="s">
-        <x:v>51</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="B10" s="16" t="n">
         <x:v>0.000945</x:v>
@@ -4694,7 +4801,7 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0">
       <x:c r="A11" s="15" t="s">
-        <x:v>52</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="B11" s="16" t="n">
         <x:v>0.0015</x:v>
@@ -4722,7 +4829,7 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0">
       <x:c r="A12" s="15" t="s">
-        <x:v>53</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="B12" s="16" t="n">
         <x:v>0.0018</x:v>
@@ -4750,7 +4857,7 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0">
       <x:c r="A13" s="15" t="s">
-        <x:v>54</x:v>
+        <x:v>16</x:v>
       </x:c>
       <x:c r="B13" s="16" t="n">
         <x:v>0.0075</x:v>
@@ -4778,7 +4885,7 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0" customHeight="1">
       <x:c r="A15" s="10" t="s">
-        <x:v>55</x:v>
+        <x:v>17</x:v>
       </x:c>
       <x:c r="B15" s="10"/>
       <x:c r="C15" s="10"/>
@@ -4789,7 +4896,7 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0">
       <x:c r="A17" s="19" t="s">
-        <x:v>56</x:v>
+        <x:v>18</x:v>
       </x:c>
       <x:c r="B17" s="19"/>
       <x:c r="C17" s="19"/>
@@ -4800,25 +4907,25 @@
     </x:row>
     <x:row r="18" ht="39.54999923706055" hidden="0">
       <x:c r="A18" s="14" t="s">
-        <x:v>57</x:v>
+        <x:v>19</x:v>
       </x:c>
       <x:c r="B18" s="14" t="s">
-        <x:v>49</x:v>
+        <x:v>11</x:v>
       </x:c>
       <x:c r="C18" s="14" t="s">
-        <x:v>50</x:v>
+        <x:v>12</x:v>
       </x:c>
       <x:c r="D18" s="14" t="s">
-        <x:v>51</x:v>
+        <x:v>13</x:v>
       </x:c>
       <x:c r="E18" s="14" t="s">
-        <x:v>52</x:v>
+        <x:v>14</x:v>
       </x:c>
       <x:c r="F18" s="14" t="s">
-        <x:v>53</x:v>
+        <x:v>15</x:v>
       </x:c>
       <x:c r="G18" s="14" t="s">
-        <x:v>54</x:v>
+        <x:v>16</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="15" hidden="0">
@@ -4980,6 +5087,9 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF5B9BD5"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="32" style="1" hidden="0" customWidth="1"/>
@@ -4987,8 +5097,8 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="17.350000381469727" hidden="0">
-      <x:c r="A1" s="2" t="s">
-        <x:v>58</x:v>
+      <x:c r="A1" s="2" t="str">
+        <x:v>Part 03: Cross-Border Ownership, Withholding and Estate Tax</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -4997,12 +5107,12 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0">
       <x:c r="A3" s="4" t="s">
-        <x:v>59</x:v>
+        <x:v>20</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0">
       <x:c r="A4" s="1" t="s">
-        <x:v>60</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="B4" s="12" t="n">
         <x:v>10000</x:v>
@@ -5010,7 +5120,7 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0">
       <x:c r="A5" s="1" t="s">
-        <x:v>61</x:v>
+        <x:v>22</x:v>
       </x:c>
       <x:c r="B5" s="13" t="n">
         <x:v>0.013</x:v>
@@ -5018,7 +5128,7 @@
     </x:row>
     <x:row r="6" ht="15" hidden="0">
       <x:c r="A6" s="1" t="s">
-        <x:v>62</x:v>
+        <x:v>23</x:v>
       </x:c>
       <x:c r="B6" s="13" t="n">
         <x:v>0.3</x:v>
@@ -5026,7 +5136,7 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0">
       <x:c r="A7" s="1" t="s">
-        <x:v>63</x:v>
+        <x:v>24</x:v>
       </x:c>
       <x:c r="B7" s="13" t="n">
         <x:v>0.15</x:v>
@@ -5035,21 +5145,21 @@
     <x:row r="9" ht="26.850000381469727" hidden="0">
       <x:c r="A9" s="14"/>
       <x:c r="B9" s="14" t="s">
-        <x:v>64</x:v>
+        <x:v>25</x:v>
       </x:c>
       <x:c r="C9" s="14" t="s">
-        <x:v>65</x:v>
+        <x:v>26</x:v>
       </x:c>
       <x:c r="D9" s="14" t="s">
-        <x:v>66</x:v>
+        <x:v>27</x:v>
       </x:c>
       <x:c r="E9" s="14" t="s">
-        <x:v>67</x:v>
+        <x:v>28</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="15" hidden="0">
       <x:c r="A10" s="15" t="s">
-        <x:v>68</x:v>
+        <x:v>29</x:v>
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f aca="0">$B$4*$B$5</x:f>
@@ -5070,7 +5180,7 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0">
       <x:c r="A11" s="15" t="s">
-        <x:v>69</x:v>
+        <x:v>30</x:v>
       </x:c>
       <x:c r="B11" s="18" t="n">
         <x:f aca="0">$B$4*$B$5</x:f>
@@ -5091,7 +5201,7 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0">
       <x:c r="A12" s="15" t="s">
-        <x:v>70</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="B12" s="22"/>
       <x:c r="C12" s="22"/>
@@ -5103,21 +5213,21 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0">
       <x:c r="A14" s="4" t="s">
-        <x:v>71</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="26.850000381469727" hidden="0">
       <x:c r="A15" s="14" t="s">
-        <x:v>72</x:v>
+        <x:v>33</x:v>
       </x:c>
       <x:c r="B15" s="14" t="s">
-        <x:v>73</x:v>
+        <x:v>34</x:v>
       </x:c>
       <x:c r="C15" s="14" t="s">
-        <x:v>74</x:v>
+        <x:v>35</x:v>
       </x:c>
       <x:c r="D15" s="14" t="s">
-        <x:v>75</x:v>
+        <x:v>36</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0">
@@ -5290,19 +5400,19 @@
     </x:row>
     <x:row r="29" ht="15" hidden="0" customHeight="1">
       <x:c r="A29" s="1" t="s">
-        <x:v>76</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B29" s="12" t="n">
         <x:v>13000</x:v>
       </x:c>
       <x:c r="D29" s="10" t="s">
-        <x:v>77</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="E29" s="10"/>
     </x:row>
     <x:row r="30" ht="15" hidden="0">
       <x:c r="A30" s="1" t="s">
-        <x:v>78</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="B30" s="24" t="n">
         <x:v>150000</x:v>
@@ -5316,7 +5426,7 @@
     </x:row>
     <x:row r="32" ht="15" hidden="0">
       <x:c r="A32" s="1" t="s">
-        <x:v>79</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="B32" s="11" t="n">
         <x:f aca="0">MATCH(B30,A16:A27)</x:f>
@@ -5327,7 +5437,7 @@
     </x:row>
     <x:row r="33" ht="15" hidden="0">
       <x:c r="A33" s="1" t="s">
-        <x:v>80</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="B33" s="25" t="n">
         <x:f aca="0">INDEX(C16:C27,B32)</x:f>
@@ -5338,7 +5448,7 @@
     </x:row>
     <x:row r="34" ht="15" hidden="0">
       <x:c r="A34" s="1" t="s">
-        <x:v>81</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="B34" s="26" t="n">
         <x:f aca="0">INDEX(D16:D27,B32)</x:f>
@@ -5347,7 +5457,7 @@
     </x:row>
     <x:row r="35" ht="15" hidden="0">
       <x:c r="A35" s="1" t="s">
-        <x:v>82</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="B35" s="27" t="n">
         <x:f aca="0">INDEX(A16:A27,B32)</x:f>
@@ -5356,7 +5466,7 @@
     </x:row>
     <x:row r="36" ht="15" hidden="0">
       <x:c r="A36" s="1" t="s">
-        <x:v>83</x:v>
+        <x:v>44</x:v>
       </x:c>
       <x:c r="B36" s="28" t="n">
         <x:f aca="0">B33+B34*(B30-B35)</x:f>
@@ -5365,7 +5475,7 @@
     </x:row>
     <x:row r="37" ht="15" hidden="0">
       <x:c r="A37" s="1" t="s">
-        <x:v>84</x:v>
+        <x:v>45</x:v>
       </x:c>
       <x:c r="B37" s="25" t="n">
         <x:f aca="0">$B$29</x:f>
@@ -5374,7 +5484,7 @@
     </x:row>
     <x:row r="38" ht="15" hidden="0">
       <x:c r="A38" s="1" t="s">
-        <x:v>85</x:v>
+        <x:v>46</x:v>
       </x:c>
       <x:c r="B38" s="28" t="n">
         <x:f aca="0">MAX(0,B36-B37)</x:f>
@@ -5383,7 +5493,7 @@
     </x:row>
     <x:row r="39" ht="15" hidden="0">
       <x:c r="A39" s="1" t="s">
-        <x:v>86</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="B39" s="11" t="str">
         <x:f aca="0">IF(B30&gt;=60000,"Yes","No")</x:f>
@@ -5401,6 +5511,9 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF70AD47"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="26" style="1" hidden="0" customWidth="1"/>
@@ -5410,8 +5523,8 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="17.350000381469727" hidden="0">
-      <x:c r="A1" s="2" t="s">
-        <x:v>87</x:v>
+      <x:c r="A1" s="2" t="str">
+        <x:v>Part 04: Portfolio Architecture and Diversification</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -5420,7 +5533,7 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0">
       <x:c r="A3" s="22" t="s">
-        <x:v>88</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="B3" s="20" t="n">
         <x:v>0.7</x:v>
@@ -5428,7 +5541,7 @@
     </x:row>
     <x:row r="4" ht="15" hidden="0">
       <x:c r="A4" s="22" t="s">
-        <x:v>89</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="B4" s="21" t="n">
         <x:f aca="0">1-B3</x:f>
@@ -5437,7 +5550,7 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0">
       <x:c r="A5" s="22" t="s">
-        <x:v>90</x:v>
+        <x:v>50</x:v>
       </x:c>
       <x:c r="B5" s="20" t="n">
         <x:v>0.16</x:v>
@@ -5445,7 +5558,7 @@
     </x:row>
     <x:row r="6" ht="15" hidden="0">
       <x:c r="A6" s="22" t="s">
-        <x:v>91</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="B6" s="20" t="n">
         <x:v>0.06</x:v>
@@ -5453,7 +5566,7 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0">
       <x:c r="A7" s="22" t="s">
-        <x:v>92</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B7" s="20" t="n">
         <x:v>0.1</x:v>
@@ -5465,7 +5578,7 @@
     </x:row>
     <x:row r="9" ht="15" hidden="0">
       <x:c r="A9" s="22" t="s">
-        <x:v>93</x:v>
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B9" s="29" t="n">
         <x:f aca="0">B3^2*B5^2+B4^2*B6^2+2*B3*B4*B7*B5*B6</x:f>
@@ -5474,7 +5587,7 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0">
       <x:c r="A10" s="22" t="s">
-        <x:v>94</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B10" s="30" t="n">
         <x:f aca="0">SQRT(B9)</x:f>
@@ -5483,7 +5596,7 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0">
       <x:c r="A11" s="22" t="s">
-        <x:v>95</x:v>
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B11" s="31" t="n">
         <x:f aca="0">B3*B5+B4*B6</x:f>
@@ -5492,7 +5605,7 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0">
       <x:c r="A12" s="22" t="s">
-        <x:v>96</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B12" s="30" t="n">
         <x:f aca="0">B11-B10</x:f>
@@ -5501,7 +5614,7 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0">
       <x:c r="A15" s="19" t="s">
-        <x:v>97</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="B15" s="19"/>
       <x:c r="C15" s="19"/>
@@ -5510,16 +5623,16 @@
     </x:row>
     <x:row r="16" ht="26.850000381469727" hidden="0">
       <x:c r="A16" s="14" t="s">
-        <x:v>92</x:v>
+        <x:v>52</x:v>
       </x:c>
       <x:c r="B16" s="14" t="s">
-        <x:v>98</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C16" s="14" t="s">
-        <x:v>99</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="D16" s="14" t="s">
-        <x:v>96</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="E16" s="14"/>
     </x:row>
@@ -5644,7 +5757,7 @@
     </x:row>
     <x:row r="26" ht="15" hidden="0">
       <x:c r="A26" s="19" t="s">
-        <x:v>100</x:v>
+        <x:v>60</x:v>
       </x:c>
       <x:c r="B26" s="19"/>
       <x:c r="C26" s="19"/>
@@ -5653,20 +5766,20 @@
     </x:row>
     <x:row r="27" ht="15" hidden="0">
       <x:c r="A27" s="14" t="s">
-        <x:v>101</x:v>
+        <x:v>61</x:v>
       </x:c>
       <x:c r="B27" s="14" t="s">
-        <x:v>102</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C27" s="14" t="s">
-        <x:v>103</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="D27" s="14"/>
       <x:c r="E27" s="14"/>
     </x:row>
     <x:row r="28" ht="15" hidden="0">
       <x:c r="A28" s="15" t="s">
-        <x:v>104</x:v>
+        <x:v>64</x:v>
       </x:c>
       <x:c r="B28" s="20" t="n">
         <x:v>0.55</x:v>
@@ -5677,7 +5790,7 @@
     </x:row>
     <x:row r="29" ht="15" hidden="0">
       <x:c r="A29" s="15" t="s">
-        <x:v>105</x:v>
+        <x:v>65</x:v>
       </x:c>
       <x:c r="B29" s="20" t="n">
         <x:v>0.15</x:v>
@@ -5688,7 +5801,7 @@
     </x:row>
     <x:row r="30" ht="15" hidden="0">
       <x:c r="A30" s="15" t="s">
-        <x:v>106</x:v>
+        <x:v>66</x:v>
       </x:c>
       <x:c r="B30" s="20" t="n">
         <x:v>0.3</x:v>
@@ -5699,7 +5812,7 @@
     </x:row>
     <x:row r="31" ht="15" hidden="0">
       <x:c r="A31" s="11" t="s">
-        <x:v>107</x:v>
+        <x:v>67</x:v>
       </x:c>
       <x:c r="B31" s="13" t="n">
         <x:v>0.1</x:v>
@@ -5707,7 +5820,7 @@
     </x:row>
     <x:row r="32" ht="15" hidden="0">
       <x:c r="A32" s="11" t="s">
-        <x:v>108</x:v>
+        <x:v>68</x:v>
       </x:c>
       <x:c r="B32" s="13" t="n">
         <x:v>0.75</x:v>
@@ -5715,7 +5828,7 @@
     </x:row>
     <x:row r="33" ht="15" hidden="0">
       <x:c r="A33" s="11" t="s">
-        <x:v>109</x:v>
+        <x:v>69</x:v>
       </x:c>
       <x:c r="B33" s="13" t="n">
         <x:v>0.05</x:v>
@@ -5723,7 +5836,7 @@
     </x:row>
     <x:row r="35" ht="15" hidden="0">
       <x:c r="A35" s="11" t="s">
-        <x:v>110</x:v>
+        <x:v>70</x:v>
       </x:c>
       <x:c r="B35" s="32" t="n">
         <x:f aca="0">B28^2*C28^2+B29^2*C29^2+B30^2*C30^2+2*B28*B29*B31*C28*C29+2*B28*B30*B32*C28*C30+2*B29*B30*B33*C29*C30</x:f>
@@ -5732,7 +5845,7 @@
     </x:row>
     <x:row r="36" ht="15" hidden="0">
       <x:c r="A36" s="4" t="s">
-        <x:v>111</x:v>
+        <x:v>71</x:v>
       </x:c>
       <x:c r="B36" s="33" t="n">
         <x:f aca="0">SQRT(B35)</x:f>
@@ -5741,7 +5854,7 @@
     </x:row>
     <x:row r="37" ht="15" hidden="0">
       <x:c r="A37" s="11" t="s">
-        <x:v>99</x:v>
+        <x:v>59</x:v>
       </x:c>
       <x:c r="B37" s="34" t="n">
         <x:f aca="0">B28*C28+B29*C29+B30*C30</x:f>
@@ -5750,7 +5863,7 @@
     </x:row>
     <x:row r="38" ht="15" hidden="0">
       <x:c r="A38" s="4" t="s">
-        <x:v>96</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B38" s="33" t="n">
         <x:f aca="0">B37-B36</x:f>
@@ -5769,17 +5882,22 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FF70AD47"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="40" style="1" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="52" style="1" hidden="0" customWidth="1"/>
     <x:col min="2" max="3" width="12" style="1" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" style="1" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="20" style="1" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16" style="1" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22" style="1" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="18" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="17.350000381469727" hidden="0">
-      <x:c r="A1" s="2" t="s">
-        <x:v>112</x:v>
+      <x:c r="A1" s="2" t="str">
+        <x:v>Part 04: Portfolio Architecture and Blended Costs</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -5788,7 +5906,7 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0">
       <x:c r="A3" s="1" t="s">
-        <x:v>113</x:v>
+        <x:v>72</x:v>
       </x:c>
       <x:c r="B3" s="12" t="n">
         <x:v>50000</x:v>
@@ -5796,24 +5914,24 @@
     </x:row>
     <x:row r="5" ht="39.54999923706055" hidden="0">
       <x:c r="A5" s="14" t="s">
-        <x:v>114</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="B5" s="14" t="s">
-        <x:v>102</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C5" s="14" t="s">
-        <x:v>43</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D5" s="14" t="s">
-        <x:v>115</x:v>
+        <x:v>74</x:v>
       </x:c>
       <x:c r="E5" s="14" t="s">
-        <x:v>116</x:v>
+        <x:v>75</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="15" hidden="0">
       <x:c r="A6" s="15" t="s">
-        <x:v>117</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B6" s="20" t="n">
         <x:v>0.55</x:v>
@@ -5832,7 +5950,7 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0">
       <x:c r="A7" s="15" t="s">
-        <x:v>118</x:v>
+        <x:v>77</x:v>
       </x:c>
       <x:c r="B7" s="20" t="n">
         <x:v>0.15</x:v>
@@ -5851,7 +5969,7 @@
     </x:row>
     <x:row r="8" ht="15" hidden="0">
       <x:c r="A8" s="15" t="s">
-        <x:v>119</x:v>
+        <x:v>78</x:v>
       </x:c>
       <x:c r="B8" s="20" t="n">
         <x:v>0.15</x:v>
@@ -5870,7 +5988,7 @@
     </x:row>
     <x:row r="9" ht="15" hidden="0">
       <x:c r="A9" s="15" t="s">
-        <x:v>120</x:v>
+        <x:v>79</x:v>
       </x:c>
       <x:c r="B9" s="20" t="n">
         <x:v>0.075</x:v>
@@ -5889,7 +6007,7 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0">
       <x:c r="A10" s="15" t="s">
-        <x:v>121</x:v>
+        <x:v>80</x:v>
       </x:c>
       <x:c r="B10" s="20" t="n">
         <x:v>0.075</x:v>
@@ -5908,7 +6026,7 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0">
       <x:c r="A11" s="35" t="s">
-        <x:v>122</x:v>
+        <x:v>81</x:v>
       </x:c>
       <x:c r="B11" s="36" t="n">
         <x:f aca="0">SUM(B6:B10)</x:f>
@@ -5926,7 +6044,7 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0">
       <x:c r="A13" s="11" t="s">
-        <x:v>123</x:v>
+        <x:v>82</x:v>
       </x:c>
       <x:c r="B13" s="28" t="n">
         <x:f aca="0">$B$3*E11</x:f>
@@ -5935,29 +6053,29 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0">
       <x:c r="A15" s="19" t="s">
-        <x:v>124</x:v>
+        <x:v>83</x:v>
       </x:c>
       <x:c r="B15" s="19"/>
       <x:c r="C15" s="19"/>
       <x:c r="D15" s="19"/>
       <x:c r="E15" s="19"/>
     </x:row>
-    <x:row r="16" ht="39.54999923706055" hidden="0">
+    <x:row r="16" ht="42" hidden="0" customHeight="1">
       <x:c r="A16" s="14" t="s">
-        <x:v>114</x:v>
+        <x:v>73</x:v>
       </x:c>
       <x:c r="B16" s="14" t="s">
-        <x:v>125</x:v>
+        <x:v>84</x:v>
       </x:c>
       <x:c r="C16" s="14" t="s">
-        <x:v>126</x:v>
+        <x:v>85</x:v>
       </x:c>
       <x:c r="D16" s="14"/>
       <x:c r="E16" s="14"/>
     </x:row>
     <x:row r="17" ht="15" hidden="0">
       <x:c r="A17" s="15" t="s">
-        <x:v>117</x:v>
+        <x:v>76</x:v>
       </x:c>
       <x:c r="B17" s="20" t="n">
         <x:v>0.35</x:v>
@@ -5968,7 +6086,7 @@
     </x:row>
     <x:row r="18" ht="15" hidden="0">
       <x:c r="A18" s="15" t="s">
-        <x:v>127</x:v>
+        <x:v>86</x:v>
       </x:c>
       <x:c r="B18" s="20" t="n">
         <x:v>0.45</x:v>
@@ -5979,7 +6097,7 @@
     </x:row>
     <x:row r="19" ht="15" hidden="0">
       <x:c r="A19" s="15" t="s">
-        <x:v>128</x:v>
+        <x:v>87</x:v>
       </x:c>
       <x:c r="B19" s="20" t="n">
         <x:v>0.05</x:v>
@@ -5990,7 +6108,7 @@
     </x:row>
     <x:row r="20" ht="15" hidden="0">
       <x:c r="A20" s="15" t="s">
-        <x:v>129</x:v>
+        <x:v>88</x:v>
       </x:c>
       <x:c r="B20" s="20" t="n">
         <x:v>0.1</x:v>
@@ -6001,7 +6119,7 @@
     </x:row>
     <x:row r="21" ht="15" hidden="0">
       <x:c r="A21" s="15" t="s">
-        <x:v>130</x:v>
+        <x:v>89</x:v>
       </x:c>
       <x:c r="B21" s="20" t="n">
         <x:v>0.05</x:v>
@@ -6012,7 +6130,7 @@
     </x:row>
     <x:row r="22" ht="15" hidden="0">
       <x:c r="A22" s="4" t="s">
-        <x:v>131</x:v>
+        <x:v>90</x:v>
       </x:c>
       <x:c r="B22" s="39" t="n">
         <x:f aca="0">B17*C6+B18*C7+B19*C8+B20*C9+B21*C10</x:f>
@@ -6034,17 +6152,20 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFFFC000"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="10" style="1" hidden="0" customWidth="1"/>
-    <x:col min="2" max="2" width="14" style="1" hidden="0" customWidth="1"/>
-    <x:col min="3" max="3" width="30" style="1" hidden="0" customWidth="1"/>
-    <x:col min="4" max="4" width="14" style="1" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="28" style="1" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="17" style="1" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="34" style="1" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="24" style="1" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="17.350000381469727" hidden="0">
-      <x:c r="A1" s="2" t="s">
-        <x:v>132</x:v>
+      <x:c r="A1" s="2" t="str">
+        <x:v>Part 05: Core Overlap and Concentration</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -6052,7 +6173,7 @@
     </x:row>
     <x:row r="2" ht="22.350000381469727" hidden="0" customHeight="1">
       <x:c r="A2" s="10" t="s">
-        <x:v>133</x:v>
+        <x:v>91</x:v>
       </x:c>
       <x:c r="B2" s="10"/>
       <x:c r="C2" s="10"/>
@@ -6060,14 +6181,14 @@
     </x:row>
     <x:row r="4" ht="15" hidden="0" customHeight="1">
       <x:c r="A4" s="14" t="s">
-        <x:v>134</x:v>
+        <x:v>92</x:v>
       </x:c>
       <x:c r="B4" s="14" t="s">
-        <x:v>102</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="C4" s="14"/>
-      <x:c r="D4" s="40" t="s">
-        <x:v>135</x:v>
+      <x:c r="D4" s="85" t="s">
+        <x:v>93</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0">
@@ -6077,7 +6198,7 @@
       <x:c r="B5" s="16" t="n">
         <x:v>0.033333</x:v>
       </x:c>
-      <x:c r="D5" s="40"/>
+      <x:c r="D5" s="85"/>
     </x:row>
     <x:row r="6" ht="15" hidden="0">
       <x:c r="A6" s="15" t="n">
@@ -6086,7 +6207,7 @@
       <x:c r="B6" s="16" t="n">
         <x:v>0.033333</x:v>
       </x:c>
-      <x:c r="D6" s="40"/>
+      <x:c r="D6" s="85"/>
     </x:row>
     <x:row r="7" ht="15" hidden="0">
       <x:c r="A7" s="15" t="n">
@@ -6095,7 +6216,7 @@
       <x:c r="B7" s="16" t="n">
         <x:v>0.033333</x:v>
       </x:c>
-      <x:c r="D7" s="40"/>
+      <x:c r="D7" s="85"/>
     </x:row>
     <x:row r="8" ht="15" hidden="0">
       <x:c r="A8" s="15" t="n">
@@ -6104,7 +6225,7 @@
       <x:c r="B8" s="16" t="n">
         <x:v>0.033333</x:v>
       </x:c>
-      <x:c r="D8" s="40"/>
+      <x:c r="D8" s="85"/>
     </x:row>
     <x:row r="9" ht="15" hidden="0">
       <x:c r="A9" s="15" t="n">
@@ -6113,7 +6234,7 @@
       <x:c r="B9" s="16" t="n">
         <x:v>0.033333</x:v>
       </x:c>
-      <x:c r="D9" s="40"/>
+      <x:c r="D9" s="85"/>
     </x:row>
     <x:row r="10" ht="15" hidden="0">
       <x:c r="A10" s="15" t="n">
@@ -6122,7 +6243,7 @@
       <x:c r="B10" s="16" t="n">
         <x:v>0.033333</x:v>
       </x:c>
-      <x:c r="D10" s="40"/>
+      <x:c r="D10" s="85"/>
     </x:row>
     <x:row r="11" ht="15" hidden="0">
       <x:c r="A11" s="15" t="n">
@@ -6131,6 +6252,7 @@
       <x:c r="B11" s="16" t="n">
         <x:v>0.033333</x:v>
       </x:c>
+      <x:c r="D11" s="88"/>
     </x:row>
     <x:row r="12" ht="15" hidden="0">
       <x:c r="A12" s="15" t="n">
@@ -6318,7 +6440,7 @@
     </x:row>
     <x:row r="36" ht="15" hidden="0">
       <x:c r="A36" s="1" t="s">
-        <x:v>136</x:v>
+        <x:v>94</x:v>
       </x:c>
       <x:c r="B36" s="26" t="n">
         <x:f aca="0">SUM(B5:B34)</x:f>
@@ -6327,7 +6449,7 @@
     </x:row>
     <x:row r="37" ht="15" hidden="0">
       <x:c r="A37" s="1" t="s">
-        <x:v>137</x:v>
+        <x:v>95</x:v>
       </x:c>
       <x:c r="B37" s="41" t="n">
         <x:f aca="0">SUMSQ(B5:B34)</x:f>
@@ -6336,7 +6458,7 @@
     </x:row>
     <x:row r="38" ht="15" hidden="0">
       <x:c r="A38" s="1" t="s">
-        <x:v>138</x:v>
+        <x:v>96</x:v>
       </x:c>
       <x:c r="B38" s="42" t="n">
         <x:f aca="0">1/B37</x:f>
@@ -6345,30 +6467,30 @@
     </x:row>
     <x:row r="39" ht="15" hidden="0">
       <x:c r="A39" s="1" t="s">
-        <x:v>139</x:v>
+        <x:v>97</x:v>
       </x:c>
       <x:c r="B39" s="11" t="n">
         <x:f aca="0">COUNTIF(B5:B34,"&gt;0")</x:f>
         <x:v>30</x:v>
       </x:c>
     </x:row>
-    <x:row r="42" ht="15" hidden="0">
-      <x:c r="A42" s="19" t="s">
-        <x:v>140</x:v>
-      </x:c>
-      <x:c r="B42" s="19"/>
-      <x:c r="C42" s="19"/>
-      <x:c r="D42" s="19"/>
+    <x:row r="42" ht="30" hidden="0" customHeight="1">
+      <x:c r="A42" s="90" t="s">
+        <x:v>98</x:v>
+      </x:c>
+      <x:c r="B42" s="90"/>
+      <x:c r="C42" s="90"/>
+      <x:c r="D42" s="90"/>
     </x:row>
     <x:row r="43" ht="26.850000381469727" hidden="0">
       <x:c r="A43" s="14" t="s">
-        <x:v>141</x:v>
+        <x:v>99</x:v>
       </x:c>
       <x:c r="B43" s="14" t="s">
-        <x:v>142</x:v>
+        <x:v>100</x:v>
       </x:c>
       <x:c r="C43" s="14" t="s">
-        <x:v>143</x:v>
+        <x:v>101</x:v>
       </x:c>
       <x:c r="D43" s="14"/>
     </x:row>
@@ -6450,26 +6572,26 @@
         <x:v>500</x:v>
       </x:c>
     </x:row>
-    <x:row r="52" ht="15" hidden="0">
-      <x:c r="A52" s="19" t="s">
-        <x:v>144</x:v>
-      </x:c>
-      <x:c r="B52" s="19"/>
-      <x:c r="C52" s="19"/>
-      <x:c r="D52" s="19"/>
+    <x:row r="52" ht="34" hidden="0" customHeight="1">
+      <x:c r="A52" s="90" t="s">
+        <x:v>102</x:v>
+      </x:c>
+      <x:c r="B52" s="90"/>
+      <x:c r="C52" s="90"/>
+      <x:c r="D52" s="90"/>
     </x:row>
     <x:row r="53" ht="39.54999923706055" hidden="0">
       <x:c r="A53" s="14" t="s">
-        <x:v>145</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="B53" s="14" t="s">
-        <x:v>146</x:v>
+        <x:v>104</x:v>
       </x:c>
       <x:c r="C53" s="14" t="s">
-        <x:v>147</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="D53" s="14" t="s">
-        <x:v>148</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="54" ht="15" hidden="0">
@@ -6605,15 +6727,22 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFED7D31"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="22" style="1" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="36" style="1" hidden="0" customWidth="1"/>
     <x:col min="2" max="5" width="12" style="1" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="17" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="17" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="17" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="17" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="17.350000381469727" hidden="0">
-      <x:c r="A1" s="2" t="s">
-        <x:v>149</x:v>
+      <x:c r="A1" s="2" t="str">
+        <x:v>Part 06: Satellite Exposure and Portfolio Risk</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -6622,26 +6751,26 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0">
       <x:c r="A3" s="4" t="s">
-        <x:v>150</x:v>
+        <x:v>107</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="26.850000381469727" hidden="0">
       <x:c r="B4" s="14" t="s">
-        <x:v>151</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="C4" s="14" t="s">
-        <x:v>152</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="D4" s="14" t="s">
-        <x:v>153</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="E4" s="14" t="s">
-        <x:v>154</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="15" hidden="0">
       <x:c r="A5" s="11" t="s">
-        <x:v>102</x:v>
+        <x:v>62</x:v>
       </x:c>
       <x:c r="B5" s="13" t="n">
         <x:v>0.55</x:v>
@@ -6658,26 +6787,26 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0">
       <x:c r="A7" s="4" t="s">
-        <x:v>155</x:v>
+        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="8" ht="26.850000381469727" hidden="0">
       <x:c r="B8" s="14" t="s">
-        <x:v>151</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="C8" s="14" t="s">
-        <x:v>152</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="D8" s="14" t="s">
-        <x:v>153</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="E8" s="14" t="s">
-        <x:v>154</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="15" hidden="0">
       <x:c r="A9" s="11" t="s">
-        <x:v>103</x:v>
+        <x:v>63</x:v>
       </x:c>
       <x:c r="B9" s="13" t="n">
         <x:v>0.16</x:v>
@@ -6694,27 +6823,27 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0">
       <x:c r="A11" s="4" t="s">
-        <x:v>156</x:v>
+        <x:v>113</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="26.850000381469727" hidden="0">
       <x:c r="A12" s="22"/>
       <x:c r="B12" s="14" t="s">
-        <x:v>151</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="C12" s="14" t="s">
-        <x:v>152</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="D12" s="14" t="s">
-        <x:v>153</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="E12" s="14" t="s">
-        <x:v>154</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="15" hidden="0">
       <x:c r="A13" s="15" t="s">
-        <x:v>151</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B13" s="20" t="n">
         <x:v>1</x:v>
@@ -6731,7 +6860,7 @@
     </x:row>
     <x:row r="14" ht="15" hidden="0">
       <x:c r="A14" s="15" t="s">
-        <x:v>152</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B14" s="20" t="n">
         <x:v>0.1</x:v>
@@ -6748,7 +6877,7 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0">
       <x:c r="A15" s="15" t="s">
-        <x:v>153</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="B15" s="20" t="n">
         <x:v>0.85</x:v>
@@ -6765,7 +6894,7 @@
     </x:row>
     <x:row r="16" ht="15" hidden="0">
       <x:c r="A16" s="15" t="s">
-        <x:v>154</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="B16" s="20" t="n">
         <x:v>0.75</x:v>
@@ -6781,28 +6910,28 @@
       </x:c>
     </x:row>
     <x:row r="18" ht="15" hidden="0">
-      <x:c r="A18" s="4" t="s">
-        <x:v>157</x:v>
+      <x:c r="A18" s="4" t="str">
+        <x:v>Covariance matrix (vol_i × vol_j × rho_ij)</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="26.850000381469727" hidden="0">
       <x:c r="A19" s="22"/>
       <x:c r="B19" s="14" t="s">
-        <x:v>151</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="C19" s="14" t="s">
-        <x:v>152</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="D19" s="14" t="s">
-        <x:v>153</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="E19" s="14" t="s">
-        <x:v>154</x:v>
+        <x:v>111</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="15" hidden="0">
       <x:c r="A20" s="15" t="s">
-        <x:v>151</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B20" s="45" t="n">
         <x:f aca="0">B$9*B$9*B13</x:f>
@@ -6823,7 +6952,7 @@
     </x:row>
     <x:row r="21" ht="15" hidden="0">
       <x:c r="A21" s="15" t="s">
-        <x:v>152</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B21" s="45" t="n">
         <x:f aca="0">C$9*B$9*B14</x:f>
@@ -6844,7 +6973,7 @@
     </x:row>
     <x:row r="22" ht="15" hidden="0">
       <x:c r="A22" s="15" t="s">
-        <x:v>153</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="B22" s="45" t="n">
         <x:f aca="0">D$9*B$9*B15</x:f>
@@ -6865,7 +6994,7 @@
     </x:row>
     <x:row r="23" ht="15" hidden="0">
       <x:c r="A23" s="15" t="s">
-        <x:v>154</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="B23" s="45" t="n">
         <x:f aca="0">E$9*B$9*B16</x:f>
@@ -6885,26 +7014,26 @@
       </x:c>
     </x:row>
     <x:row r="25" ht="15" hidden="0">
-      <x:c r="A25" s="4" t="s">
-        <x:v>158</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26" ht="15" hidden="0" customHeight="1">
-      <x:c r="A26" s="11" t="s">
-        <x:v>93</x:v>
+      <x:c r="A25" s="4" t="str">
+        <x:v>Portfolio variance (full double-sum expansion of wᵀΣw)</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26" ht="24" hidden="0" customHeight="1">
+      <x:c r="A26" s="77" t="s">
+        <x:v>53</x:v>
       </x:c>
       <x:c r="B26" s="46" t="n">
         <x:f aca="0">$B$5*$B$5*B20+$B$5*$C$5*C20+$B$5*$D$5*D20+$B$5*$E$5*E20+$C$5*$B$5*B21+$C$5*$C$5*C21+$C$5*$D$5*D21+$C$5*$E$5*E21+$D$5*$B$5*B22+$D$5*$C$5*C22+$D$5*$D$5*D22+$D$5*$E$5*E22+$E$5*$B$5*B23+$E$5*$C$5*C23+$E$5*$D$5*D23+$E$5*$E$5*E23</x:f>
         <x:v>0.023186500000000002</x:v>
       </x:c>
       <x:c r="D26" s="10" t="s">
-        <x:v>159</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="E26" s="10"/>
     </x:row>
-    <x:row r="27" ht="15" hidden="0">
-      <x:c r="A27" s="4" t="s">
-        <x:v>94</x:v>
+    <x:row r="27" ht="24" hidden="0" customHeight="1">
+      <x:c r="A27" s="90" t="s">
+        <x:v>54</x:v>
       </x:c>
       <x:c r="B27" s="33" t="n">
         <x:f aca="0">SQRT(B26)</x:f>
@@ -6913,9 +7042,9 @@
       <x:c r="D27" s="10"/>
       <x:c r="E27" s="10"/>
     </x:row>
-    <x:row r="28" ht="15" hidden="0">
-      <x:c r="A28" s="11" t="s">
-        <x:v>95</x:v>
+    <x:row r="28" ht="24" hidden="0" customHeight="1">
+      <x:c r="A28" s="77" t="s">
+        <x:v>55</x:v>
       </x:c>
       <x:c r="B28" s="34" t="n">
         <x:f aca="0">B$5*B$9+C$5*C$9+D$5*D$9+E$5*E$9</x:f>
@@ -6926,7 +7055,7 @@
     </x:row>
     <x:row r="29" ht="15" hidden="0">
       <x:c r="A29" s="4" t="s">
-        <x:v>96</x:v>
+        <x:v>56</x:v>
       </x:c>
       <x:c r="B29" s="33" t="n">
         <x:f aca="0">B28-B27</x:f>
@@ -6946,27 +7075,32 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFC55A11"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="30" style="1" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="52" style="1" hidden="0" customWidth="1"/>
     <x:col min="2" max="3" width="14" style="1" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="19" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="18" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="17.350000381469727" hidden="0">
-      <x:c r="A1" s="2" t="s">
-        <x:v>160</x:v>
+      <x:c r="A1" s="2" t="str">
+        <x:v>Part 07: Options Income as a Tactical Sleeve</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
     </x:row>
     <x:row r="3" ht="15" hidden="0">
       <x:c r="A3" s="4" t="s">
-        <x:v>161</x:v>
+        <x:v>115</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0">
       <x:c r="A4" s="22" t="s">
-        <x:v>162</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="B4" s="47" t="n">
         <x:v>100</x:v>
@@ -6974,7 +7108,7 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0">
       <x:c r="A5" s="22" t="s">
-        <x:v>163</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="B5" s="47" t="n">
         <x:v>90</x:v>
@@ -6982,7 +7116,7 @@
     </x:row>
     <x:row r="6" ht="15" hidden="0">
       <x:c r="A6" s="22" t="s">
-        <x:v>164</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="B6" s="47" t="n">
         <x:v>2</x:v>
@@ -6990,7 +7124,7 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0">
       <x:c r="A7" s="22" t="s">
-        <x:v>165</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B7" s="43" t="n">
         <x:v>1</x:v>
@@ -7002,7 +7136,7 @@
     </x:row>
     <x:row r="9" ht="15" hidden="0">
       <x:c r="A9" s="22" t="s">
-        <x:v>166</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B9" s="18" t="n">
         <x:f aca="0">B5*100*B7</x:f>
@@ -7011,7 +7145,7 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0">
       <x:c r="A10" s="22" t="s">
-        <x:v>167</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f aca="0">B6*100*B7</x:f>
@@ -7020,7 +7154,7 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0">
       <x:c r="A11" s="22" t="s">
-        <x:v>168</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="B11" s="18" t="n">
         <x:f aca="0">B5-B6</x:f>
@@ -7029,7 +7163,7 @@
     </x:row>
     <x:row r="12" ht="15" hidden="0">
       <x:c r="A12" s="22" t="s">
-        <x:v>169</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="B12" s="30" t="n">
         <x:f aca="0">B10/B9</x:f>
@@ -7038,7 +7172,7 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0">
       <x:c r="A13" s="22" t="s">
-        <x:v>170</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="B13" s="21" t="n">
         <x:f aca="0">B12*12</x:f>
@@ -7046,13 +7180,13 @@
       </x:c>
     </x:row>
     <x:row r="16" ht="15" hidden="0">
-      <x:c r="A16" s="4" t="s">
-        <x:v>171</x:v>
+      <x:c r="A16" s="4" t="str">
+        <x:v>Stage 2: If assigned → covered call</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="15" hidden="0">
       <x:c r="A17" s="22" t="s">
-        <x:v>172</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B17" s="18" t="n">
         <x:f aca="0">B11</x:f>
@@ -7061,7 +7195,7 @@
     </x:row>
     <x:row r="18" ht="15" hidden="0">
       <x:c r="A18" s="22" t="s">
-        <x:v>173</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="B18" s="47" t="n">
         <x:v>95</x:v>
@@ -7069,7 +7203,7 @@
     </x:row>
     <x:row r="19" ht="15" hidden="0">
       <x:c r="A19" s="22" t="s">
-        <x:v>174</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="B19" s="47" t="n">
         <x:v>1.5</x:v>
@@ -7077,7 +7211,7 @@
     </x:row>
     <x:row r="20" ht="15" hidden="0">
       <x:c r="A20" s="22" t="s">
-        <x:v>175</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="B20" s="18" t="n">
         <x:f aca="0">B18+B19</x:f>
@@ -7086,7 +7220,7 @@
     </x:row>
     <x:row r="21" ht="15" hidden="0">
       <x:c r="A21" s="22" t="s">
-        <x:v>176</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="B21" s="37" t="n">
         <x:f aca="0">B20-B17</x:f>
@@ -7095,7 +7229,7 @@
     </x:row>
     <x:row r="22" ht="15" hidden="0">
       <x:c r="A22" s="22" t="s">
-        <x:v>177</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="B22" s="37" t="n">
         <x:f aca="0">B21*100*B7</x:f>
@@ -7104,7 +7238,7 @@
     </x:row>
     <x:row r="23" ht="15" hidden="0">
       <x:c r="A23" s="22" t="s">
-        <x:v>178</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B23" s="30" t="n">
         <x:f aca="0">B21/B17</x:f>
@@ -7113,12 +7247,12 @@
     </x:row>
     <x:row r="25" ht="15" hidden="0">
       <x:c r="A25" s="4" t="s">
-        <x:v>179</x:v>
+        <x:v>132</x:v>
       </x:c>
     </x:row>
     <x:row r="26" ht="15" hidden="0">
       <x:c r="A26" s="22" t="s">
-        <x:v>180</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="B26" s="48" t="n">
         <x:v>70</x:v>
@@ -7126,7 +7260,7 @@
     </x:row>
     <x:row r="27" ht="15" hidden="0">
       <x:c r="A27" s="22" t="s">
-        <x:v>181</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="B27" s="18" t="n">
         <x:f aca="0">B17-B26</x:f>
@@ -7135,7 +7269,7 @@
     </x:row>
     <x:row r="28" ht="15" hidden="0">
       <x:c r="A28" s="22" t="s">
-        <x:v>182</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="B28" s="37" t="n">
         <x:f aca="0">B27*100*B7</x:f>
@@ -7144,7 +7278,7 @@
     </x:row>
     <x:row r="29" ht="15" hidden="0">
       <x:c r="A29" s="22" t="s">
-        <x:v>183</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="B29" s="18" t="n">
         <x:f aca="0">B10</x:f>
@@ -7153,7 +7287,7 @@
     </x:row>
     <x:row r="30" ht="15" hidden="0">
       <x:c r="A30" s="22" t="s">
-        <x:v>184</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="B30" s="37" t="n">
         <x:f aca="0">B29-B28</x:f>
@@ -7162,20 +7296,20 @@
     </x:row>
     <x:row r="33" ht="15" hidden="0">
       <x:c r="A33" s="19" t="s">
-        <x:v>185</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="B33" s="19"/>
       <x:c r="C33" s="19"/>
     </x:row>
     <x:row r="34" ht="26.850000381469727" hidden="0">
       <x:c r="A34" s="14" t="s">
-        <x:v>186</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="B34" s="14" t="s">
-        <x:v>187</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="C34" s="14" t="s">
-        <x:v>188</x:v>
+        <x:v>141</x:v>
       </x:c>
     </x:row>
     <x:row r="35" ht="15" hidden="0">
@@ -7237,6 +7371,9 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetPr>
+    <x:tabColor rgb="FFC55A11"/>
+  </x:sheetPr>
   <x:sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15"/>
   <x:cols>
     <x:col min="1" max="1" width="34" style="1" hidden="0" customWidth="1"/>
@@ -7244,8 +7381,8 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="17.350000381469727" hidden="0">
-      <x:c r="A1" s="2" t="s">
-        <x:v>189</x:v>
+      <x:c r="A1" s="2" t="str">
+        <x:v>Part 07: Tax, Asset Location and Realized Gains</x:v>
       </x:c>
       <x:c r="B1" s="2"/>
       <x:c r="C1" s="2"/>
@@ -7253,12 +7390,12 @@
     </x:row>
     <x:row r="3" ht="15" hidden="0">
       <x:c r="A3" s="4" t="s">
-        <x:v>190</x:v>
+        <x:v>142</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="15" hidden="0">
       <x:c r="A4" s="22" t="s">
-        <x:v>191</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="B4" s="23" t="n">
         <x:v>1000</x:v>
@@ -7266,7 +7403,7 @@
     </x:row>
     <x:row r="5" ht="15" hidden="0">
       <x:c r="A5" s="22" t="s">
-        <x:v>192</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="B5" s="20" t="n">
         <x:v>0.15</x:v>
@@ -7274,7 +7411,7 @@
     </x:row>
     <x:row r="6" ht="15" hidden="0">
       <x:c r="A6" s="22" t="s">
-        <x:v>193</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="B6" s="20" t="n">
         <x:v>0.24</x:v>
@@ -7282,7 +7419,7 @@
     </x:row>
     <x:row r="7" ht="15" hidden="0">
       <x:c r="A7" s="22" t="s">
-        <x:v>194</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="B7" s="18" t="n">
         <x:f aca="0">B4*B5</x:f>
@@ -7291,7 +7428,7 @@
     </x:row>
     <x:row r="8" ht="15" hidden="0">
       <x:c r="A8" s="22" t="s">
-        <x:v>195</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="B8" s="18" t="n">
         <x:f aca="0">B4*B6</x:f>
@@ -7300,7 +7437,7 @@
     </x:row>
     <x:row r="9" ht="15" hidden="0">
       <x:c r="A9" s="22" t="s">
-        <x:v>196</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="B9" s="18" t="n">
         <x:f aca="0">B4-B7</x:f>
@@ -7309,7 +7446,7 @@
     </x:row>
     <x:row r="10" ht="15" hidden="0">
       <x:c r="A10" s="22" t="s">
-        <x:v>197</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="B10" s="18" t="n">
         <x:f aca="0">B4-B8</x:f>
@@ -7318,7 +7455,7 @@
     </x:row>
     <x:row r="11" ht="15" hidden="0">
       <x:c r="A11" s="22" t="s">
-        <x:v>198</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B11" s="37" t="n">
         <x:f aca="0">B8-B7</x:f>
@@ -7327,12 +7464,12 @@
     </x:row>
     <x:row r="13" ht="15" hidden="0">
       <x:c r="A13" s="4" t="s">
-        <x:v>199</x:v>
+        <x:v>151</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="15" hidden="0">
       <x:c r="A14" s="22" t="s">
-        <x:v>200</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="B14" s="43" t="n">
         <x:v>100</x:v>
@@ -7340,7 +7477,7 @@
     </x:row>
     <x:row r="15" ht="15" hidden="0">
       <x:c r="A15" s="22" t="s">
-        <x:v>201</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="B15" s="47" t="n">
         <x:v>50</x:v>
@@ -7348,7 +7485,7 @@
     </x:row>
     <x:row r="16" ht="15" hidden="0">
       <x:c r="A16" s="22" t="s">
-        <x:v>202</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="B16" s="47" t="n">
         <x:v>40</x:v>
@@ -7356,7 +7493,7 @@
     </x:row>
     <x:row r="17" ht="15" hidden="0">
       <x:c r="A17" s="22" t="s">
-        <x:v>203</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="B17" s="18" t="n">
         <x:f aca="0">(B15-B16)*B14</x:f>
@@ -7365,7 +7502,7 @@
     </x:row>
     <x:row r="18" ht="15" hidden="0">
       <x:c r="A18" s="22" t="s">
-        <x:v>204</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="B18" s="47" t="n">
         <x:v>41</x:v>
@@ -7373,7 +7510,7 @@
     </x:row>
     <x:row r="19" ht="15" hidden="0">
       <x:c r="A19" s="22" t="s">
-        <x:v>205</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="B19" s="43" t="n">
         <x:v>100</x:v>
@@ -7381,7 +7518,7 @@
     </x:row>
     <x:row r="20" ht="15" hidden="0">
       <x:c r="A20" s="22" t="s">
-        <x:v>206</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="B20" s="18" t="n">
         <x:f aca="0">B17*(B19/B14)</x:f>
@@ -7390,7 +7527,7 @@
     </x:row>
     <x:row r="21" ht="15" hidden="0">
       <x:c r="A21" s="22" t="s">
-        <x:v>207</x:v>
+        <x:v>159</x:v>
       </x:c>
       <x:c r="B21" s="18" t="n">
         <x:f aca="0">B17-B20</x:f>
@@ -7399,7 +7536,7 @@
     </x:row>
     <x:row r="22" ht="15" hidden="0">
       <x:c r="A22" s="22" t="s">
-        <x:v>208</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="B22" s="18" t="n">
         <x:f aca="0">B18*B19</x:f>
@@ -7408,7 +7545,7 @@
     </x:row>
     <x:row r="23" ht="15" hidden="0">
       <x:c r="A23" s="22" t="s">
-        <x:v>209</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="B23" s="37" t="n">
         <x:f aca="0">B22+B20</x:f>
@@ -7417,7 +7554,7 @@
     </x:row>
     <x:row r="24" ht="15" hidden="0">
       <x:c r="A24" s="22" t="s">
-        <x:v>210</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="B24" s="37" t="n">
         <x:f aca="0">B23/B19</x:f>
@@ -7426,23 +7563,23 @@
     </x:row>
     <x:row r="26" ht="15" hidden="0">
       <x:c r="A26" s="4" t="s">
-        <x:v>211</x:v>
+        <x:v>163</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="15" hidden="0" customHeight="1">
       <x:c r="A27" s="22" t="s">
-        <x:v>212</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="B27" s="49" t="n">
         <x:v>100000</x:v>
       </x:c>
       <x:c r="D27" s="10" t="s">
-        <x:v>213</x:v>
+        <x:v>165</x:v>
       </x:c>
     </x:row>
     <x:row r="28" ht="15" hidden="0">
       <x:c r="A28" s="22" t="s">
-        <x:v>214</x:v>
+        <x:v>166</x:v>
       </x:c>
       <x:c r="B28" s="49" t="n">
         <x:v>50000</x:v>
@@ -7451,7 +7588,7 @@
     </x:row>
     <x:row r="29" ht="15" hidden="0">
       <x:c r="A29" s="22" t="s">
-        <x:v>215</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B29" s="23" t="n">
         <x:v>49450</x:v>
@@ -7460,7 +7597,7 @@
     </x:row>
     <x:row r="30" ht="15" hidden="0">
       <x:c r="A30" s="22" t="s">
-        <x:v>216</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="B30" s="23" t="n">
         <x:v>545500</x:v>
@@ -7469,7 +7606,7 @@
     </x:row>
     <x:row r="31" ht="15" hidden="0">
       <x:c r="A31" s="22" t="s">
-        <x:v>217</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="B31" s="50" t="n">
         <x:f aca="0">B27+B28</x:f>
@@ -7479,7 +7616,7 @@
     </x:row>
     <x:row r="32" ht="15" hidden="0">
       <x:c r="A32" s="22" t="s">
-        <x:v>218</x:v>
+        <x:v>170</x:v>
       </x:c>
       <x:c r="B32" s="50" t="n">
         <x:f aca="0">MAX(0,MIN(B31,B29)-MAX(B27,0))</x:f>
@@ -7489,7 +7626,7 @@
     </x:row>
     <x:row r="33" ht="15" hidden="0">
       <x:c r="A33" s="22" t="s">
-        <x:v>219</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="B33" s="50" t="n">
         <x:f aca="0">MAX(0,MIN(B31,B30)-MAX(B27,B29))</x:f>
@@ -7499,7 +7636,7 @@
     </x:row>
     <x:row r="34" ht="15" hidden="0">
       <x:c r="A34" s="22" t="s">
-        <x:v>220</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="B34" s="50" t="n">
         <x:f aca="0">MAX(0,B31-MAX(B27,B30))</x:f>
@@ -7508,7 +7645,7 @@
     </x:row>
     <x:row r="35" ht="15" hidden="0">
       <x:c r="A35" s="22" t="s">
-        <x:v>221</x:v>
+        <x:v>173</x:v>
       </x:c>
       <x:c r="B35" s="37" t="n">
         <x:f aca="0">B32*0+B33*0.15+B34*0.2</x:f>
@@ -7517,7 +7654,7 @@
     </x:row>
     <x:row r="36" ht="15" hidden="0">
       <x:c r="A36" s="22" t="s">
-        <x:v>222</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="B36" s="36" t="n">
         <x:f aca="0">B35/B28</x:f>

</xml_diff>